<commit_message>
Import 14 new destinations from the updated spreadsheet; add endurance_event category
Updated docs/permits_worldwide_database.xlsx (117 rows, up from 102) added
15 new destinations. Munro Bagging is skipped - the spreadsheet's own
research note flags it as not fitting the model (no permit/registration
exists at all). The remaining 14 are imported as unpublished stubs via a
one-off script with hand-picked classification per row, using the new
research_notes column for the raw research text instead of the old
placeholder-translation workaround.

6 of the 14 are mass-participation registration events (closed-road
cycling sportives, multi-day walking marches) that don't fit any existing
category, so adds a new "endurance_event" Category value across backend
enum, DB enum (migration), and frontend (icon, label, filters, admin form).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NhGjrpjavTyjTwfLdUgRRX
</commit_message>
<xml_diff>
--- a/docs/permits_worldwide_database.xlsx
+++ b/docs/permits_worldwide_database.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="530">
   <si>
     <t xml:space="preserve">מדינה/אזור</t>
   </si>
@@ -935,13 +935,13 @@
     <t xml:space="preserve">Everest - היתר טיפוס לפסגה</t>
   </si>
   <si>
-    <t xml:space="preserve">עלות גבוהה, לא תחרות מכסה</t>
-  </si>
-  <si>
-    <t xml:space="preserve">היתר יקר (11,000$+), לא מכסה קשיחה אלא בירוקרטיה+עלות - פחות מתאים למודל 'הרשמה תחרותית'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">נמוכה (לא תחרותי)</t>
+    <t xml:space="preserve">עלות גבוהה + דרישת ניסיון מוכח (חדש)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">חוק חדש (עבר את הבית העליון בפרלמנט הנפאלי, טרם נכנס לתוקף מלא - צפוי אחרי בחירות מרץ 2026): מטפסים חייבים להציג אישור רשמי (לא תמונה/סקרינשוט) על סיכום פסגה של לפחות 7,000 מ' בנפאל לפני קבלת היתר לאוורסט. זו דוגמה מצוינת לשכבת 'דרישות כלליות' - לא מסמך פשוט אלא ניסיון מוכח שצריך לתכנן שנים מראש. גם מדריך נפאלי מוסמך חובה (לא מדריכים זרים), טיפוס יחיד אסור.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">נמוכה (עלות) אך גבוהה (הכנה נדרשת)</t>
   </si>
   <si>
     <t xml:space="preserve">וייטנאם</t>
@@ -1368,6 +1368,216 @@
   </si>
   <si>
     <t xml:space="preserve">ממשלתי-מלכותי (Royal Collection Trust)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">סקוטלנד/בריטניה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אירוע חצייה שנתי (עם תהליך קבלה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TGO Challenge - חצייה רגלית של סקוטלנד מים לים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">תאריך שנתי קבוע + עדיפויות + FCFS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הרשמה שנתית נפתחת בסוף ספטמבר/תחילת אוקטובר. כ-400 מקומות בסה"כ. שכבת עדיפות ראשונה (הרשמה מוקדמת מובטחת) למאמתי מסלול, מתנדבים, ומי שהשלים 10/20/30 חציות - נפתחת כשבוע לפני כולם. שאר הנרשמים - כל הקודם זוכה בתאריך ומועד קבועים (לרוב תחילת אוקטובר בצהריים). מחייב מילוי טופס ניסיון/כישורים שעובר הערכה (לא לוטו, אבל לא מובטח קבלה אוטומטית). דמי הרשמה כ-110 ליש"ט לאדם. האירוע עצמו במאי, 15 יום, מסלול אישי בין 180-200 מייל.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tgochallenge.com - מארגן: מגזין The Great Outdoors + עמותת Challenge Trust</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nijmegen Four Days Marches (Vierdaagse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מכסה עירונית קשיחה + עדיפויות + הגרלה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אירוע ההליכה הגדול בעולם - 45,000+ משתתפים, 30-50 ק"מ ליום, 4 ימים ברצף. העירייה קבעה תקרת משתתפים קשיחה. שכבת עדיפות ראשונה: מי שהשלים את המצעד לפחות פעם אחת ב-10 השנים האחרונות (הרשמה מוקדמת מובטחת). שאר הנרשמים - הגרלה. הרשמה נפתחת בינואר, האירוע במחצית יולי. לא מתחרים על זמן (non-competitive) - בדיוק כמו TGO Challenge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4daagse.nl - הכי גדול בקטגוריה הזו בעולם, שווה יעד דגל</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מסחרי/עמותה (Stichting 4Daagse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">בריטניה (וויילס)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אירוע חצייה רב-יומי (הרים)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dragon's Back Race (וויילס)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הרשמה מוגבלת + הערכת ניסיון</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מסלול הרים קשה לאורך כל וויילס, 5 ימים. הרשמה מוגבלת במספר, לעיתים דורשת תיעוד ניסיון קודם באירועי הרים דומים. שים לב: זה גבולי בין 'אירוע לא-תחרותי' לבין 'ריצת אולטרה עם תזמון' - יש בו גם מרכיב תחרותי (יש מנצחים), לשקול אם זה מתאים למודל או שייך לקטגוריית המירוצים שהוחרגה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">לאמת סטטוס הרשמה עדכני</t>
+  </si>
+  <si>
+    <t xml:space="preserve">בריטניה (סקוטלנד)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אתגר לא-רשמי (ללא הרשמה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Munro Bagging - רשימת ה-Munros הסקוטיים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אין הרשמה/היתר בכלל</t>
+  </si>
+  <si>
+    <t xml:space="preserve">עלייה ל-282 פסגות מעל 3,000 רגל בסקוטלנד - אין שום תהליך הרשמה או מכסה, זו רשימת יעדים אישית ולא אירוע מאורגן. מוסיף כדוגמה שלילית - חשוב להבדיל בין 'אתגר מפורסם' ל'אתגר עם הרשמה בפועל'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אין תחרות/הרשמה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">לא רלוונטי למודל - אין permit/הרשמה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">לא נדרש</t>
+  </si>
+  <si>
+    <t xml:space="preserve">רכיבת אופניים בכביש סגור (לא-תחרותי)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L'Étape du Tour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הרשמה מוגבלת (הגרלה/מכירה מהירה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">רוכבים חובבים על קטע אמיתי ממסלול הטור דה פראנס, כבישים סגורים לחלוטין לתנועה - יחיד מסוגו. כ-16,000 נרשמים, נגמר מהר. חלק מהשנים דרך הגרלה (ballot), חלק במכירה ישירה שנגמרת תוך ימים. הרשמה נפתחת סביב ינואר-פברואר לאירוע ביולי.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">letapedutour.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מסחרי (ASO - מארגני הטור דה פראנס)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Etape Loch Ness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">עדיפות + הרשמה כללית</t>
+  </si>
+  <si>
+    <t xml:space="preserve">66 מייל סביב לוך נס, כבישים סגורים לחלוטין. יש 'הרשמה מוקדמת מועדפת' למי שהשתתף/תרם בעבר, לפני פתיחה כללית. נגמר מהר יחסית לגודל האירוע.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">etapelochness.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Marmotte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הרשמה מהירה, נגמר תוך ימים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אחד מאירועי הרכיבה ההרריים הוותיקים והיוקרתיים באירופה (עולה לאלפ ד'הואז), נגמר מהר במיוחד גם עם עליית מחירים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">לאמת תאריך הרשמה מדויק</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Enchantments (וושינגטון)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הגרלה שנתית + הגרלה יומית בעונה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אזור Alpine Lakes Wilderness. הגרלה מתקדמת בפברואר (odds כ-3-5% לאזור הליבה), ועוד הגרלה יומית מקומית מאי-אוקטובר. מהתחרותיים ביותר בארה"ב.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">קמפינג (מכסה יומית קשיחה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kalalau Trail / Nāpali Coast (קאווואי, הוואי)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">חלון נגלל 90 יום + מכסה יומית</t>
+  </si>
+  <si>
+    <t xml:space="preserve">רק 60 מקומות ליום, נפתח 90 יום מראש בחצות (שעון הוואי), נגמר תוך פחות מ-30 שניות בעונת שיא - אחד המהירים ביותר להיגמר בעולם</t>
+  </si>
+  <si>
+    <t xml:space="preserve">explore.hawaii.gov (DLNR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Subway (זיון נפ״ל)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הגרלה חודשית</t>
+  </si>
+  <si>
+    <t xml:space="preserve">נפרד מ-Angels Landing - הגרלה חודשית דרך recreation.gov לחלון תאריכים של 3 חודשים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lake O'Hara (יוהו נפ״ל, קנדה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אחוזי זכייה נמוכים מאוד (כ-5%), גישה לאגם מוגבלת לאוטובוס רשמי או הליכה ארוכה, permit נפרד מ-West Coast Trail שכבר ברשימה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parks Canada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">קמפינג/טרק (הגרלה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grand Canyon - Corridor Backcountry Permit (Phantom Ranch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הגרלה חודשית נפרדת מהרפטינג</t>
+  </si>
+  <si>
+    <t xml:space="preserve">לינה בתחתית הקניון (לא ריין-ריבר), הגרלה נפרדת מהיתר הרפטינג שכבר ברשימה, גם היא תחרותית מאוד</t>
+  </si>
+  <si>
+    <t xml:space="preserve">recreation.gov - נפרד מ-Grand Canyon Rafting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">קמפינג (חלון נגלל)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conundrum Hot Springs (קולורדו)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מעיינות חמים פופולריים ביותר בקולורדו, הזמנה מראש חובה, נגמר מהר בקיץ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אוגנדה/טנזניה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">צפייה בעדינה (מכסה יומית)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">טרק שימפנזים (Kibale/Mahale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מקביל לגורילות אך פחות יקר ותחרותי - עדיין permit מוגבל ליום שכדאי להזמין מראש בעונת שיא</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ארגנטינה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">טיפוס (מכסה+עונתיות)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aconcagua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מכסת מטפסים + עונתיות קשיחה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הפסגה הגבוהה ביותר באמריקה מחוץ להימלאיה, permit דרך מחוז מנדוסה, מכסת מטפסים יומית/עונתית ומחיר עולה ככל שמתקרבים לשיא העונה</t>
   </si>
   <si>
     <t xml:space="preserve">הסבר</t>
@@ -1622,15 +1832,15 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1886,7 +2096,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H118"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
@@ -4499,6 +4709,394 @@
       </c>
       <c r="H103" s="3" t="s">
         <v>448</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A104" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="B104" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="F104" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G104" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="H104" s="3" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="B105" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="E105" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="F105" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G105" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="H105" s="3" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="B106" s="9" t="s">
+        <v>461</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="F106" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G106" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="H106" s="3" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A107" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="B107" s="9" t="s">
+        <v>467</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="F107" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="G107" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="H107" s="3" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A108" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B108" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="E108" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="F108" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G108" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="H108" s="3" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="B109" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="E109" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="F109" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G109" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="H109" s="3" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A110" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B110" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="E110" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="F110" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G110" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="H110" s="3" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A111" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B111" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="E111" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="F111" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G111" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H111" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A112" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B112" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="E112" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="F112" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G112" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="H112" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A113" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B113" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="E113" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="F113" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G113" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H113" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A114" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="B114" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="D114" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E114" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="F114" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G114" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="H114" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A115" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B115" s="8" t="s">
+        <v>502</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="E115" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="F115" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G115" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="H115" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A116" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B116" s="9" t="s">
+        <v>507</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E116" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G116" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H116" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A117" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="B117" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E117" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="F117" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G117" s="3"/>
+      <c r="H117" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="B118" s="9" t="s">
+        <v>515</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="E118" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G118" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="H118" s="12" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -4525,63 +5123,63 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>449</v>
+      <c r="B1" s="13" t="s">
+        <v>519</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
-        <v>450</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>451</v>
+      <c r="A2" s="14" t="s">
+        <v>520</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>521</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>452</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>453</v>
+      <c r="A3" s="14" t="s">
+        <v>522</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>523</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>454</v>
+      <c r="B4" s="12" t="s">
+        <v>524</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>455</v>
+      <c r="B5" s="12" t="s">
+        <v>525</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13"/>
-      <c r="B6" s="14"/>
+      <c r="A6" s="14"/>
+      <c r="B6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>456</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>457</v>
+      <c r="A7" s="14" t="s">
+        <v>526</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
-        <v>458</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>459</v>
+      <c r="A8" s="14" t="s">
+        <v>528</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>529</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Import 6 new destinations from the 2026-09-02 spreadsheet update
Cross-checked all 122 rows against the 116 destinations already in
the DB (handling abbreviations, diacritics, parentheticals) - only 6
were genuinely new: GR20 (Corsica), Denali NP camping (distinct from
the existing climbing permit), McNeil River and Katmai Brooks Falls
bear viewing (Alaska), Skomer Island puffins, and San Ignacio Lagoon
gray whales. Everything else in the sheet already matches an existing
row. Munro Bagging skipped again (no real permit exists). All 6 are
unpublished stubs pending the research pipeline, same as prior imports.
</commit_message>
<xml_diff>
--- a/docs/permits_worldwide_database.xlsx
+++ b/docs/permits_worldwide_database.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="556">
   <si>
     <t xml:space="preserve">מדינה/אזור</t>
   </si>
@@ -1578,6 +1578,84 @@
   </si>
   <si>
     <t xml:space="preserve">הפסגה הגבוהה ביותר באמריקה מחוץ להימלאיה, permit דרך מחוז מנדוסה, מכסת מטפסים יומית/עונתית ומחיר עולה ככל שמתקרבים לשיא העונה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ארה"ב (אלסקה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denali NP - קמפינג (Wonder Lake / Teklanika)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הזמנת קמפינג + כרטיסי אוטובוס השאטל בתוך הפארק (הכביש הפנימי סגור לרכב פרטי) - מוזמן דרך recreation.gov, נגמר מהר בעונת הקיץ הקצרה (יוני-ספטמבר). נפרד מהיתר הטיפוס לפסגה שכבר קיים בטבלה.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">צפייה בעדינה (הגרלה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">McNeil River State Game Sanctuary - צפייה בדובים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">כ-1 מתוך 10 מגישים זוכה. 185 היתרי 'Guided Viewing' + 57 היתרי 'Camp-Standby' בשנה, לתקופות של 4 ימים בין 7 ביוני ל-25 באוגוסט. הגשה עד 1 במרץ, דמי הגשה 30$ (לא מוחזרים) + דמי היתר בנפרד אם זוכים (225-525$ לפי תושבות).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adfg.alaska.gov - Alaska Department of Fish and Game</t>
+  </si>
+  <si>
+    <t xml:space="preserve">צפייה בעדינה (מעורב)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Katmai NP - Brooks Falls (צפייה בדובים)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">חלון נגלל (קמפינג) + הגרלה (הלודג')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">המקום המפורסם בעולם לצפייה בדובים תופסים סלמון קופץ. הקמפינג הממשלתי (Brooks Camp, עד 60 איש) מוזמן דרך recreation.gov כמו קמפינג רגיל. לינה בלודג' הפרטי (Brooks Lodge) מבוססת הגרלה נפרדת ויקרה (כ-1,150$/לילה). ביקור יומי בלי לינה - פחות תחרותי.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">גבוהה (ללודג'), בינונית (לקמפינג)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nps.gov/katm + katmailand.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ממשלתי (קמפינג) / מסחרי (הלודג')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ויילס (בריטניה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">צפייה בעדינה - ציפורים (מכסה יומית)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skomer Island - צפייה בפפינים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">תאריך פתיחה שנתי קבוע (1 בדצמבר)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מכסה קשיחה של 250 מבקרים ליום, עונה אפריל-ספטמבר. כרטיסים לעונה כולה נפתחים ב-1 בדצמבר מדי שנה ונגמרים תוך חודשים - שיא הביקוש: שלושת השבועות הראשונים של יוני. מפעיל סירה מורשה יחיד בלבד.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visitskomer.co.uk / pembrokeshire-islands.co.uk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מסחרי/עמותה (Wildlife Trust of South &amp; West Wales)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">צפייה בעדינה (לווייתנים - מכסת סירות)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Ignacio Lagoon - לווייתני אפור</t>
+  </si>
+  <si>
+    <t xml:space="preserve">רישוי מפעילים + מכסת סירות בו-זמנית</t>
+  </si>
+  <si>
+    <t xml:space="preserve">שמורת ביוספרה El Vizcaíno (אונסק"ו). 26 פנגות מורשות בסה"כ, מקסימום 16-20 בו-זמנית בשמורה. עונה: דצמבר-אפריל (שיא: פברואר-מרץ). מכסת מפעילים, לא הרשמה אישית ישירה - דומה במנגנון ל-Sipadan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONANP (מקסיקו) - NOM-131-SEMARNAT-2010</t>
   </si>
   <si>
     <t xml:space="preserve">הסבר</t>
@@ -2096,7 +2174,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H118"/>
+  <dimension ref="A1:H123"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
@@ -5096,6 +5174,136 @@
         <v>330</v>
       </c>
       <c r="H118" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="B119" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E119" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G119" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H119" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="B120" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="D120" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E120" s="3" t="s">
+        <v>524</v>
+      </c>
+      <c r="F120" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G120" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="H120" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="B121" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="E121" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="F121" s="3" t="s">
+        <v>530</v>
+      </c>
+      <c r="G121" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="H121" s="3" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="B122" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="E122" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="F122" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G122" s="3" t="s">
+        <v>538</v>
+      </c>
+      <c r="H122" s="3" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="B123" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="E123" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="F123" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G123" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="H123" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -5127,23 +5335,23 @@
         <v>3</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>519</v>
+        <v>545</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>520</v>
+        <v>546</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>521</v>
+        <v>547</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>522</v>
+        <v>548</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>523</v>
+        <v>549</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5151,7 +5359,7 @@
         <v>102</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>524</v>
+        <v>550</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5159,7 +5367,7 @@
         <v>44</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>525</v>
+        <v>551</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5168,18 +5376,18 @@
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>526</v>
+        <v>552</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>527</v>
+        <v>553</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>528</v>
+        <v>554</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>529</v>
+        <v>555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>